<commit_message>
Auto update: 2026-06-16 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -459,11 +459,22 @@
         <v>397242</v>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t>（内容由AI生成，仅供参考）</t>
         </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>396957</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: 2026-06-17 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -477,6 +477,19 @@
         <v>396957</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>396171</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-786</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-06-18 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -490,6 +490,19 @@
         <v>-786</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>394267</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-1904</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-06-21 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -503,6 +503,19 @@
         <v>-1904</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>395012</v>
+      </c>
+      <c r="C8" t="n">
+        <v>745</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-06-23 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -516,6 +516,19 @@
         <v>745</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>393937</v>
+      </c>
+      <c r="C9" t="n">
+        <v>-1075</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-06-24 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -529,6 +529,19 @@
         <v>-1075</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>392910</v>
+      </c>
+      <c r="C10" t="n">
+        <v>-1027</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-06-25 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -542,6 +542,19 @@
         <v>-1027</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>388956</v>
+      </c>
+      <c r="C11" t="n">
+        <v>-3954</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-06-26 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -555,6 +555,19 @@
         <v>-3954</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>385191</v>
+      </c>
+      <c r="C12" t="n">
+        <v>-3765</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-06-27 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -568,6 +568,19 @@
         <v>-3765</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>382084</v>
+      </c>
+      <c r="C13" t="n">
+        <v>-3107</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-06-30 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -581,6 +581,19 @@
         <v>-3107</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>380534</v>
+      </c>
+      <c r="C14" t="n">
+        <v>-1550</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-02 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -594,6 +594,19 @@
         <v>-1550</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>375079</v>
+      </c>
+      <c r="C15" t="n">
+        <v>-5455</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-03 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -607,6 +607,19 @@
         <v>-5455</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>373018</v>
+      </c>
+      <c r="C16" t="n">
+        <v>-2061</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-08 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -620,6 +620,19 @@
         <v>-2061</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>362466</v>
+      </c>
+      <c r="C17" t="n">
+        <v>-10552</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-09 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -633,6 +633,19 @@
         <v>-10552</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>354261</v>
+      </c>
+      <c r="C18" t="n">
+        <v>-8205</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-10 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -646,6 +646,19 @@
         <v>-8205</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>346419</v>
+      </c>
+      <c r="C19" t="n">
+        <v>-7842</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-11 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -659,6 +659,19 @@
         <v>-7842</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>344269</v>
+      </c>
+      <c r="C20" t="n">
+        <v>-2150</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-14 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -672,6 +672,19 @@
         <v>-2150</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>342574</v>
+      </c>
+      <c r="C21" t="n">
+        <v>-1695</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-15 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -685,6 +685,19 @@
         <v>-1695</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>339652</v>
+      </c>
+      <c r="C22" t="n">
+        <v>-2922</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-16 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -698,6 +698,19 @@
         <v>-2922</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>334289</v>
+      </c>
+      <c r="C23" t="n">
+        <v>-5363</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-17 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -711,6 +711,19 @@
         <v>-5363</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>334254</v>
+      </c>
+      <c r="C24" t="n">
+        <v>-35</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-18 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -724,6 +724,19 @@
         <v>-35</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>332945</v>
+      </c>
+      <c r="C25" t="n">
+        <v>-1309</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-21 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -737,6 +737,19 @@
         <v>-1309</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>329870</v>
+      </c>
+      <c r="C26" t="n">
+        <v>-3075</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-22 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -750,6 +750,19 @@
         <v>-3075</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>328759</v>
+      </c>
+      <c r="C27" t="n">
+        <v>-1111</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-23 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -763,6 +763,19 @@
         <v>-1111</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>320615</v>
+      </c>
+      <c r="C28" t="n">
+        <v>-8144</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-24 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -776,6 +776,19 @@
         <v>-8144</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>315883</v>
+      </c>
+      <c r="C29" t="n">
+        <v>-4732</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-25 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -789,6 +789,19 @@
         <v>-4732</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>311317</v>
+      </c>
+      <c r="C30" t="n">
+        <v>-4566</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-28 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -802,6 +802,19 @@
         <v>-4566</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>292810</v>
+      </c>
+      <c r="C31" t="n">
+        <v>-18507</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-29 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -815,6 +815,19 @@
         <v>-18507</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>289759</v>
+      </c>
+      <c r="C32" t="n">
+        <v>-3051</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-30 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -828,6 +828,19 @@
         <v>-3051</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>274168</v>
+      </c>
+      <c r="C33" t="n">
+        <v>-15591</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-07-31 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -841,6 +841,19 @@
         <v>-15591</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>266204</v>
+      </c>
+      <c r="C34" t="n">
+        <v>-7964</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-08-02 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -854,6 +854,19 @@
         <v>-7964</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>264179</v>
+      </c>
+      <c r="C35" t="n">
+        <v>-2025</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-08-04 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -867,6 +867,19 @@
         <v>-2025</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>260720</v>
+      </c>
+      <c r="C36" t="n">
+        <v>-3459</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-08-06 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -880,6 +880,19 @@
         <v>-3459</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>251417</v>
+      </c>
+      <c r="C37" t="n">
+        <v>-9303</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-08-07 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -893,6 +893,19 @@
         <v>-9303</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>248897</v>
+      </c>
+      <c r="C38" t="n">
+        <v>-2520</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-08-08 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -906,6 +906,19 @@
         <v>-2520</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>244172</v>
+      </c>
+      <c r="C39" t="n">
+        <v>-4725</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-08-11 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -919,6 +919,19 @@
         <v>-4725</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>242673</v>
+      </c>
+      <c r="C40" t="n">
+        <v>-1499</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-08-12 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -932,6 +932,19 @@
         <v>-1499</v>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>241838</v>
+      </c>
+      <c r="C41" t="n">
+        <v>-835</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-08-13 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -945,6 +945,19 @@
         <v>-835</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>240285</v>
+      </c>
+      <c r="C42" t="n">
+        <v>-1553</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-08-14 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -958,6 +958,19 @@
         <v>-1553</v>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>236430</v>
+      </c>
+      <c r="C43" t="n">
+        <v>-3855</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-08-15 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -971,6 +971,19 @@
         <v>-3855</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>231445</v>
+      </c>
+      <c r="C44" t="n">
+        <v>-4985</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-08-18 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -984,6 +984,19 @@
         <v>-4985</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>231340</v>
+      </c>
+      <c r="C45" t="n">
+        <v>-105</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-08-19 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -997,6 +997,19 @@
         <v>-105</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>229214</v>
+      </c>
+      <c r="C46" t="n">
+        <v>-2126</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-08-21 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1010,6 +1010,19 @@
         <v>-2126</v>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>228378</v>
+      </c>
+      <c r="C47" t="n">
+        <v>-836</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-08-22 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1023,6 +1023,19 @@
         <v>-836</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>227992</v>
+      </c>
+      <c r="C48" t="n">
+        <v>-386</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-08-25 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1036,6 +1036,19 @@
         <v>-386</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>226242</v>
+      </c>
+      <c r="C49" t="n">
+        <v>-1750</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-08-26 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1049,6 +1049,19 @@
         <v>-1750</v>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>225442</v>
+      </c>
+      <c r="C50" t="n">
+        <v>-800</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-08-27 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1062,6 +1062,19 @@
         <v>-800</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>224011</v>
+      </c>
+      <c r="C51" t="n">
+        <v>-1431</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-08-28 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1075,6 +1075,19 @@
         <v>-1431</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>223976</v>
+      </c>
+      <c r="C52" t="n">
+        <v>-35</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-09-01 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1088,6 +1088,19 @@
         <v>-35</v>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>223976</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-09-02 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1101,6 +1101,19 @@
         <v>0</v>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>223911</v>
+      </c>
+      <c r="C54" t="n">
+        <v>-65</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-09-03 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1114,6 +1114,19 @@
         <v>-65</v>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>223762</v>
+      </c>
+      <c r="C55" t="n">
+        <v>-149</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-09-04 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1127,6 +1127,19 @@
         <v>-149</v>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>223712</v>
+      </c>
+      <c r="C56" t="n">
+        <v>-50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-09-05 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1140,6 +1140,19 @@
         <v>-50</v>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>223712</v>
+      </c>
+      <c r="C57" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-09-09 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1153,6 +1153,19 @@
         <v>0</v>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>218838</v>
+      </c>
+      <c r="C58" t="n">
+        <v>-4874</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-09-10 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1166,6 +1166,19 @@
         <v>-4874</v>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>220452</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1614</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-09-11 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1179,6 +1179,19 @@
         <v>1614</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>218457</v>
+      </c>
+      <c r="C60" t="n">
+        <v>-1995</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-09-12 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1192,6 +1192,19 @@
         <v>-1995</v>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>217932</v>
+      </c>
+      <c r="C61" t="n">
+        <v>-525</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>